<commit_message>
feat: Enhance conversation investigation package with PCAP support
- Updated package.json to include PCAP metadata and download ID.
- Added new PCAP file and metadata CSV for conversation investigation.
- Modified SIP trace CSV to include additional fields for better tracking.
- Enhanced timeline CSV to reflect updated SIP message details.
- Updated PowerShell script to handle new API invocations for SIP traces and PCAP downloads.
- Improved integration tests to validate new features and ensure correct API interactions.
- Updated task plan to reflect completion of PCAP export functionality.
</commit_message>
<xml_diff>
--- a/samples/demo-conversation-investigation/demo-conversation-investigation.xlsx
+++ b/samples/demo-conversation-investigation/demo-conversation-investigation.xlsx
@@ -7,6 +7,7 @@
     <sheet name="Timeline" sheetId="3" r:id="rId3"/>
     <sheet name="SIP Trace" sheetId="4" r:id="rId4"/>
     <sheet name="Evidence" sheetId="5" r:id="rId5"/>
+    <sheet name="PCAP Metadata" sheetId="6" r:id="rId6"/>
   </sheets>
 </workbook>
 </file>
@@ -75,11 +76,16 @@
           <t>SipMessages</t>
         </is>
       </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>PcapDownloaded</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-07T17:15:17.1851141Z</t>
+          <t>2026-05-07T17:45:46.2239290Z</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -135,6 +141,11 @@
       <c r="L2" t="inlineStr">
         <is>
           <t>3</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>True</t>
         </is>
       </c>
     </row>
@@ -434,7 +445,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>&lt;sip:+15551230000@example.invalid&gt;</t>
+          <t>+15551230000</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -464,7 +475,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>StartLine=INVITE sip:+15559870000@example.invalid SIP/2.0; CallID=demo-call-001; CSeq=1 INVITE; UserAgent=Demo WebRTC Client; MediaIP=203.0.113.10; AudioPort=19000; MediaDirection=sendrecv</t>
+          <t>StartLine=INVITE; CallID=demo-call-001; CSeq=1 INVITE; UserAgent=Demo WebRTC Client; SourceIP=203.0.113.10; SourcePort=19000</t>
         </is>
       </c>
     </row>
@@ -491,7 +502,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>&lt;sip:+15551230000@example.invalid&gt;</t>
+          <t>+15551230000</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -548,7 +559,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>&lt;sip:+15551230000@example.invalid&gt;</t>
+          <t>+15551230000</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -913,6 +924,36 @@
           <t>MediaDirection</t>
         </is>
       </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>SourceIP</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>SourcePort</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>DestinationIP</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>DestinationPort</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>CorrelationID</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>ConversationId</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -932,12 +973,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Request</t>
+          <t>Metadata</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>INVITE sip:+15559870000@example.invalid SIP/2.0</t>
+          <t>INVITE</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -962,17 +1003,17 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>&lt;sip:+15551230000@example.invalid&gt;</t>
+          <t>+15551230000</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>&lt;sip:+15559870000@example.invalid&gt;</t>
+          <t>+15559870000</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>&lt;sip:demo.agent@example.invalid&gt;</t>
+          <t>demo.agent@example.invalid</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -992,22 +1033,52 @@
       </c>
       <c r="P2" t="inlineStr">
         <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
           <t>203.0.113.10</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr">
+      <c r="U2" t="inlineStr">
         <is>
           <t>19000</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>0 8 101</t>
-        </is>
-      </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>sendrecv</t>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>demo-conversation-001</t>
         </is>
       </c>
     </row>
@@ -1059,12 +1130,12 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>&lt;sip:+15551230000@example.invalid&gt;</t>
+          <t>+15551230000</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>&lt;sip:+15559870000@example.invalid&gt;</t>
+          <t>+15559870000</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -1105,6 +1176,36 @@
       <c r="S3" t="inlineStr">
         <is>
           <t/>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>demo-conversation-001</t>
         </is>
       </c>
     </row>
@@ -1156,12 +1257,12 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>&lt;sip:+15551230000@example.invalid&gt;</t>
+          <t>+15551230000</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>&lt;sip:+15559870000@example.invalid&gt;</t>
+          <t>+15559870000</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -1202,6 +1303,36 @@
       <c r="S4" t="inlineStr">
         <is>
           <t/>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>demo-conversation-001</t>
         </is>
       </c>
     </row>
@@ -1227,12 +1358,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>participants</t>
+          <t>conversationLookup</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>{"userId":"demo-agent-001","purpose":"agent"}</t>
+          <t>{"id":"demo-conversation-001","startTime":"2026-05-01T14:00:00Z","endTime":"2026-05-01T14:12:45Z"}</t>
         </is>
       </c>
     </row>
@@ -1244,67 +1375,354 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{"userId":"demo-customer-001","purpose":"customer"}</t>
+          <t>{"userId":"demo-agent-001","purpose":"agent"}</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>agents</t>
+          <t>participants</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>{"id":"demo-agent-001","name":"Demo Agent","email":"demo.agent@example.invalid","state":"ACTIVE"}</t>
+          <t>{"userId":"demo-customer-001","purpose":"customer"}</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>divisions</t>
+          <t>agents</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>{"id":"demo-agent-001","division":{"id":"demo-division","name":"CustomerCare"}}</t>
+          <t>{"id":"demo-agent-001","name":"Demo Agent","email":"demo.agent@example.invalid","state":"ACTIVE"}</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>skills</t>
+          <t>divisions</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>{"id":"demo-skill-voice","name":"Voice Support","state":"active"}</t>
+          <t>{"id":"demo-agent-001","division":{"id":"demo-division","name":"CustomerCare"}}</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>recordings</t>
+          <t>skills</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>{"id":"demo-recording-001","conversationId":"demo-conversation-001","mediaType":"audio"}</t>
+          <t>{"id":"demo-skill-voice","name":"Voice Support","state":"active"}</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>recordings</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>{"id":"demo-recording-001","conversationId":"demo-conversation-001","mediaType":"audio"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
           <t>evaluations</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>{"id":"demo-evaluation-001","conversation":{"id":"demo-conversation-001"},"totalScore":91}</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>method</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>callid</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>fromUser</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>toUser</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>contactUser</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>userAgent</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>cseq</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>via1</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>sourceIp</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>sourcePort</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>conversationId</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>replyReason</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-05-01T14:00:20.000Z</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>INVITE</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>demo-call-001</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>+15551230000</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>+15559870000</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>demo.agent@example.invalid</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Demo WebRTC Client</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>1 INVITE</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>SIP/2.0/TLS edge.example.invalid</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>203.0.113.10</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>19000</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>demo-conversation-001</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-05-01T14:00:25.000Z</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>demo-call-001</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>+15551230000</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>+15559870000</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Demo Edge</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>1 INVITE</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>SIP/2.0/TLS edge.example.invalid</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>demo-conversation-001</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>180 Ringing</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-05-01T14:00:30.000Z</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>demo-call-001</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>+15551230000</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>+15559870000</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Demo SBC</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>1 INVITE</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>SIP/2.0/TLS edge.example.invalid</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>demo-conversation-001</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>486 Busy Here</t>
         </is>
       </c>
     </row>

</xml_diff>